<commit_message>
Add sector comparison for Voice Agent demand and 7 new-sector leads
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H2nHrh8216Rrq5Lnjq6sAe
</commit_message>
<xml_diff>
--- a/leads/voice-agent-leads-2026-09.xlsx
+++ b/leads/voice-agent-leads-2026-09.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="Sıcak Lead (doğrulanmış)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Karar Vericiler (LinkedIn)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tüm Liste (255)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Nasıl kullanılır" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sektör Analizi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tüm Liste (255)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Nasıl kullanılır" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sıcak Lead (doğrulanmış)'!$A$1:$S$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Karar Vericiler (LinkedIn)'!$A$1:$O$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tüm Liste (255)'!$A$1:$O$256</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tüm Liste (255)'!$A$1:$O$256</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +39,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -75,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -89,6 +94,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4078,6 +4095,845 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Sektör (İstanbul)</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>taranan işletme</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>'ulaşamadım' sinyali olan</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>oran</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>toplam yorum</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>yorum</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="n"/>
+      <c r="I1" s="3" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Oto servis / bayi</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>%17</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>2680</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>En güçlü sinyal: bayilerde çağrı yükü yüksek, randevu ve parça fiyatı telefonla soruluyor.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Sürücü kursu</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>%17</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>4806</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Kayıt dönemlerinde yoğun arama; kaçan çağrı = kaçan kayıt.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Araç kiralama</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>%8</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>2224</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>7/24 acil ve rezervasyon aramaları; çok dilli (turist) ihtiyaç.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Butik otel</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>%8</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>13313</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Rezervasyon ve yabancı misafir aramaları; çok dilli ihtiyaç.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Emlak ofisi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>%8</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>1223</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>İlan başına çok sayıda arama, danışman sahada olduğu için açılamıyor.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Restoran (rezervasyon)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>%0</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>64483</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Çok yorum var ama şikâyetler yemek/servis üzerine; telefon sinyali çıkmadı.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Veteriner</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>%0</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2593</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Sinyal çıkmadı; yine de mesai dışı acil arama potansiyeli var.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Fizik tedavi</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>%0</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>788</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Sinyal çıkmadı; randevu tabanlı, küçük örneklem.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Nakliyat</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>%0</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>563</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Sinyal çıkmadı; teklif talebi telefonla geliyor, küçük örneklem.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Pilates stüdyosu</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>%0</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>532</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Sinyal çıkmadı; mesajla (Inboxly) daha uygun.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Kuaför</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>%0</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Sinyal çıkmadı; randevular çoğunlukla WhatsApp/Instagram → Inboxly.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Avukatlık bürosu</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>%0</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>143</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Yorum çok az, ölçülemedi.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Karşılaştırma: Klinikler (önceki tarama)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>255</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>%7</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Daha geniş tarama (26 kelime) ile ~%7 işletmede doğrulanmış sinyal.</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Yeni sektörlerden sıcak lead'ler</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>sektör</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>işletme</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>öncelik</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>telefon</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>puan</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>yorum sayısı</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>kanıt (yorum özeti)</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>maps linki</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>oto servis</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Toyota Plaza Kar</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>+90 212 567 22 22</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.toyotakar.com.tr/</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>1046</v>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>2023–2026 arası 6 şikâyet: telefonlara bakılmıyor, 25 dk bekletip cevap yok, randevu alınamıyor, 'kaç gündür telefonlar açılmıyor' (Mar 2026). Yetkili bayi → bütçe var.</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Toyota%20Plaza%20Kar&amp;query_place_id=ChIJg-BM1o67yhQRA9D27m2_MUc</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>oto servis</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>otoedirnekapı</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>+90 212 531 30 06</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>http://otoedirnekapi.com.tr/</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>520</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Parça fiyatı sormak için arayanlara telefon açılmıyor, WhatsApp'a dönülmüyor (2018, 2021, 2022).</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=otoedirnekap%C4%B1&amp;query_place_id=ChIJTUBpMxG6yhQRJS3aTRFopPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>sürücü kursu</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>İstanbul Marmara Sürücü Kursu</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>+90 212 631 59 99</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>http://www.marmaraehliyet.com/</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>357</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Kayıt olmak isteyen aday aramış, kimse açmamış — doğrudan kayıp müşteri.</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=%C4%B0stanbul%20Marmara%20S%C3%BCr%C3%BCc%C3%BC%20Kursu&amp;query_place_id=ChIJweJZaSK6yhQR_rbOFjtuwyw</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>sürücü kursu</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Özel Kadıköy Ekip Sürücü Kursu</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>+90 216 346 11 16</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>http://www.ekipsurucukursu.com/</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>489</v>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Kayıt sonrası 'bilgilendireceğiz' denmiş, geri dönüş yapılmamış.</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=%C3%96zel%20Kad%C4%B1k%C3%B6y%20Ekip%20S%C3%BCr%C3%BCc%C3%BC%20Kursu&amp;query_place_id=ChIJx3ufBWa4yhQRI7NMWXMVTrw</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>araç kiralama</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Garenta İstanbul Haliç Araç Kiralama</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>+90 212 945 94 21</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.garenta.com/tr</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>1320</v>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Acil durumda ulaşılamıyor, defalarca aransa da dönüş yok (Nis 2025). Ulusal marka şubesi.</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Garenta%20%C4%B0stanbul%20Hali%C3%A7%20Ara%C3%A7%20Kiralama&amp;query_place_id=ChIJQxwa5327yhQRTYsNEWskACw</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>butik otel</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Pasaport Pier Istanbul</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>+90 216 450 22 23</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>https://istanbulpasaportpier.com/</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>566</v>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Otele telefonla ulaşmak imkansız (2023).</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Pasaport%20Pier%20Istanbul&amp;query_place_id=ChIJU1bNmn65yhQRHc_TCkOpAr0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>emlak ofisi</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>SULUKULE GAYRİMENKUL</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>+90 549 353 05 51</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>http://www.sulukuleemlak.com/</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Telefona bakmıyor, geri dönmüyor (2023).</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=SULUKULE%20GAYR%C4%B0MENKUL&amp;query_place_id=ChIJHwz_MxS6yhQRRsC0j7gE34s</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Her sektörde sadece 12 işletme ve 8 anahtar kelime tarandı (bütçe sınırı). Sıfır çıkan sektörlerde ihtiyaç yok demek değildir; örneklem küçüktür. Sıralama yön göstericidir.</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -18816,7 +19672,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>